<commit_message>
Fix dual and relaxed integer
</commit_message>
<xml_diff>
--- a/Lectures/Ex2-1Dual.xlsx
+++ b/Lectures/Ex2-1Dual.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Box\_Rosenberg2024\Classes\CEE6410\Fall2024\CEE6410-Rosenberg-GitHub\CEE-6410-Rosenberg\Lectures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F18F206-8268-402C-8C82-7A0E8CC975DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{51BE297C-7159-4B7F-A8B4-EDEB9E5D7394}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{55395D80-39AC-451B-A160-2F09F4DD3438}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DEECCA6F-6AC2-48DC-AFF3-13F33E6A024A}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of Contents" sheetId="11" r:id="rId1"/>
@@ -51,6 +51,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
@@ -604,7 +607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32FFAB76-4932-4993-B56F-965F4B099A6A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE47236B-3DCC-4D7C-9347-EF4E263148E8}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -848,26 +851,26 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" location="A!A1" display="A" xr:uid="{EB293F61-3BA2-4CC3-856C-F1C9AF7E70B8}"/>
-    <hyperlink ref="A3" location="b!A1" display="b" xr:uid="{F7C9BA0B-D2D8-4B3C-A4D7-5B4D16147D45}"/>
-    <hyperlink ref="A4" location="c!A1" display="c" xr:uid="{D412A30F-16CA-47BD-9953-114370573CAA}"/>
-    <hyperlink ref="A5" location="plnt!A1" display="plnt" xr:uid="{09978CD7-6C86-40F4-B71F-5A138D253B75}"/>
-    <hyperlink ref="A6" location="Scalar!A1" display="PROFIT_PRIMAL" xr:uid="{9A9482F5-C5D0-4349-AECC-C3A726A096F3}"/>
-    <hyperlink ref="A7" location="Scalar!A1" display="REDCOST_DUAL" xr:uid="{C06EB510-9A1D-456E-A839-32D4C3262B91}"/>
-    <hyperlink ref="A8" location="res!A1" display="res" xr:uid="{1A6D8F10-2050-4232-A35E-CEBA9C79562A}"/>
-    <hyperlink ref="A9" location="RES_CONS_DUAL!A1" display="RES_CONS_DUAL" xr:uid="{B537FEA6-9BE2-415B-A899-87054F8B7981}"/>
-    <hyperlink ref="A10" location="RES_CONS_PRIMAL!A1" display="RES_CONS_PRIMAL" xr:uid="{B9130B72-8C91-407D-9408-CFDD1581DA6E}"/>
-    <hyperlink ref="A11" location="Scalar!A1" display="VPROFIT" xr:uid="{C38A48D0-693C-4076-B7EC-E7FAE4456713}"/>
-    <hyperlink ref="A12" location="Scalar!A1" display="VREDCOST" xr:uid="{2CE72C73-944B-4FDB-8B4F-38BABC982DF4}"/>
-    <hyperlink ref="A13" location="X!A1" display="X" xr:uid="{7242153B-A89C-4C8B-801F-1DF0ED414AA4}"/>
-    <hyperlink ref="A14" location="Y!A1" display="Y" xr:uid="{52785FCF-21A0-4CA2-B7C3-ABA836BA9267}"/>
+    <hyperlink ref="A2" location="A!A1" display="A" xr:uid="{E606F7B4-2146-4158-9CC0-554B12141064}"/>
+    <hyperlink ref="A3" location="b!A1" display="b" xr:uid="{AA953FD1-AFB5-42B0-B9F5-8512D785F3A2}"/>
+    <hyperlink ref="A4" location="c!A1" display="c" xr:uid="{95E41494-595D-41B2-83D5-6BBD43A1BE20}"/>
+    <hyperlink ref="A5" location="plnt!A1" display="plnt" xr:uid="{D17157D9-9D15-4F4A-B4E6-22E5550119BE}"/>
+    <hyperlink ref="A6" location="Scalar!A1" display="PROFIT_PRIMAL" xr:uid="{565561DB-20BD-4717-AAD0-DD513CA45D84}"/>
+    <hyperlink ref="A7" location="Scalar!A1" display="REDCOST_DUAL" xr:uid="{B4F1CCC2-EC36-45BC-8D58-0E3CEDC3BF41}"/>
+    <hyperlink ref="A8" location="res!A1" display="res" xr:uid="{3F4FE753-2736-4CCB-8174-77794E296BDE}"/>
+    <hyperlink ref="A9" location="RES_CONS_DUAL!A1" display="RES_CONS_DUAL" xr:uid="{36DDDA93-83C4-45DA-B866-F8369456D226}"/>
+    <hyperlink ref="A10" location="RES_CONS_PRIMAL!A1" display="RES_CONS_PRIMAL" xr:uid="{30B6993D-E5A4-4845-8B85-3F262A07196C}"/>
+    <hyperlink ref="A11" location="Scalar!A1" display="VPROFIT" xr:uid="{2BF2233F-F966-461C-95AB-EDF049598E80}"/>
+    <hyperlink ref="A12" location="Scalar!A1" display="VREDCOST" xr:uid="{6F3CBD03-7382-485E-9565-F2440A4DDFEC}"/>
+    <hyperlink ref="A13" location="X!A1" display="X" xr:uid="{E68F4D95-717B-49B5-822B-6CE88D92CB2A}"/>
+    <hyperlink ref="A14" location="Y!A1" display="Y" xr:uid="{90ACBA0A-3519-4819-A9C1-1C207EF6323D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264387A5-D1AD-43C1-9BE3-9D73BEFB30F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF55AC60-4CCF-4A91-8EE4-EBEB3E58D4C8}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -912,7 +915,7 @@
         <v>16</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C4">
         <v>2400</v>
@@ -929,7 +932,7 @@
         <v>17</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C5">
         <v>800</v>
@@ -942,16 +945,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{264387A5-D1AD-43C1-9BE3-9D73BEFB30F8}"/>
+  <autoFilter ref="A3:E5" xr:uid="{DF55AC60-4CCF-4A91-8EE4-EBEB3E58D4C8}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{0A5D5ECC-1678-4D44-A020-89982902342D}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{8193CD49-DE14-4414-A23E-26C78686DDAD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1194DA1A-E4A0-46C0-9BDA-A9C8DDE080AC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B2CA415-2572-4E3E-8D38-B9D241990BA9}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1043,16 +1046,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E6" xr:uid="{1194DA1A-E4A0-46C0-9BDA-A9C8DDE080AC}"/>
+  <autoFilter ref="A3:E6" xr:uid="{5B2CA415-2572-4E3E-8D38-B9D241990BA9}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{02A98083-2655-450D-ACFB-7929992DA705}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{A838C05C-0676-41FD-A3F5-8AF36CFFE756}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C88C0006-4563-4AF9-9A1F-BAFEC5A972A1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D792406A-764B-47C9-86A8-AF02662E6E73}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1194,14 +1197,14 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{A234E4BA-C68C-4214-BEF4-16177079C1EB}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{C9E9A348-CEEB-4C2D-9096-7EA2A3C9104A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66966E53-41EF-487F-90D5-8ED885A1E833}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C73574DB-6E41-4BD9-B399-103A7497C193}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1302,16 +1305,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:C9" xr:uid="{66966E53-41EF-487F-90D5-8ED885A1E833}"/>
+  <autoFilter ref="A3:C9" xr:uid="{C73574DB-6E41-4BD9-B399-103A7497C193}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{2235FDC7-3A5A-486D-B636-2D9E2E38FFAD}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{AECFC37C-B520-4E3B-9517-6A62D3C0A525}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2723F353-3ED7-4090-BC3C-E35103488DD1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F85A7E-7B7A-41D4-9F8A-DE38521D757A}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1367,16 +1370,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B6" xr:uid="{2723F353-3ED7-4090-BC3C-E35103488DD1}"/>
+  <autoFilter ref="A3:B6" xr:uid="{F7F85A7E-7B7A-41D4-9F8A-DE38521D757A}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{12FA5008-70D9-4F10-9076-95E3ED044FBF}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{941A18F2-180D-4440-BEA8-E82A9BF2D482}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48A324A2-8F58-458E-85ED-34D864DCF718}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67387396-820B-4DB0-B16E-30DB68D184C7}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1424,16 +1427,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B5" xr:uid="{48A324A2-8F58-458E-85ED-34D864DCF718}"/>
+  <autoFilter ref="A3:B5" xr:uid="{67387396-820B-4DB0-B16E-30DB68D184C7}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{90455C30-5A2D-4298-B595-99EA3F888361}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{3CC41C78-D1E4-4DBC-915C-B00438125825}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1917BF81-B106-41E8-8B1E-EA8A6B3717AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90F90EE4-01E2-46E6-8FCA-5B012F159C10}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1472,16 +1475,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:A5" xr:uid="{1917BF81-B106-41E8-8B1E-EA8A6B3717AB}"/>
+  <autoFilter ref="A3:A5" xr:uid="{90F90EE4-01E2-46E6-8FCA-5B012F159C10}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{5A612B21-A4F7-40C0-983D-46C330EBC0B6}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{4A023336-7230-44D5-BD47-4162EE9BF47A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3452BC93-E6A3-48D4-BF82-ED18DF1E7F7F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{005999E6-F57E-4DF6-9353-762437821221}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1525,16 +1528,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:A6" xr:uid="{3452BC93-E6A3-48D4-BF82-ED18DF1E7F7F}"/>
+  <autoFilter ref="A3:A6" xr:uid="{005999E6-F57E-4DF6-9353-762437821221}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{D35C7154-D62A-4C96-ABDE-5D604A77F31A}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{38922720-007D-4B2E-839D-A605FBAF7F4D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20ECEB7F-D50E-46B1-9FE0-A8D8EA04D123}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D6E9B8D-E1C0-40AF-9580-6FE23C1B1E02}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1609,16 +1612,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E5" xr:uid="{20ECEB7F-D50E-46B1-9FE0-A8D8EA04D123}"/>
+  <autoFilter ref="A3:E5" xr:uid="{6D6E9B8D-E1C0-40AF-9580-6FE23C1B1E02}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{85F28717-E61C-4BE0-B52D-8F2940DE7BE2}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{83C11B53-71EC-4800-9AA9-0A47CDD11DBF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A259D38-1633-4A3F-8934-3924E6F1C484}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F64716E-A11C-4507-83CB-9CED2AC25A91}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1710,9 +1713,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E6" xr:uid="{9A259D38-1633-4A3F-8934-3924E6F1C484}"/>
+  <autoFilter ref="A3:E6" xr:uid="{3F64716E-A11C-4507-83CB-9CED2AC25A91}"/>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{02546A90-3376-4EEC-B241-41AA3D9A090E}"/>
+    <hyperlink ref="A1" location="'Table of Contents'!A1" display="TOC" xr:uid="{FE303A1F-E95B-4A1F-8E7D-0E1D86D8DA9E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>